<commit_message>
Fix SKLU1952893 location LCH01 -> LCH04 via CORRECTIONS.csv
Adds CORRECTIONS.csv (Container No. + Booking No. -> Location) applied
before calculation; the change is recorded in the Remark column and the
source files stay untouched. Reruns KMBK 2611N (LCH) with the fix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATABASE/STORAGE_DATABASE.xlsx
+++ b/DATABASE/STORAGE_DATABASE.xlsx
@@ -770,7 +770,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>ESCO B3 / LCMT A0/B1</t>
+          <t>LCMT A0/B1</t>
         </is>
       </c>
       <c r="K3" s="4" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>04/10/2026 09:05</t>
+          <t>04/10/2026 09:47</t>
         </is>
       </c>
     </row>
@@ -31878,17 +31878,17 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>LCH01</t>
+          <t>LCH04</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>ESCO B3</t>
+          <t>LCMT A0/B1</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -31991,7 +31991,11 @@
       <c r="AL206" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="AM206" s="2" t="n"/>
+      <c r="AM206" s="2" t="inlineStr">
+        <is>
+          <t>แก้ Location LCH01 → LCH04 (CORRECTIONS.csv: ตู้เข้า LCMT จริงตาม GATE และ BKG LWharf (LOAD/B/L ระบุ LCH01))</t>
+        </is>
+      </c>
       <c r="AN206" s="2" t="inlineStr">
         <is>
           <t>Kanokporn</t>

</xml_diff>